<commit_message>
QA: Actualizacion de la matriz de registro de control de versiones con hashes de commits y ramas reales
</commit_message>
<xml_diff>
--- a/Matriz de registro(MODELO DE CONTROL DE VERSIONES).xlsx
+++ b/Matriz de registro(MODELO DE CONTROL DE VERSIONES).xlsx
@@ -1915,7 +1915,7 @@
       </c>
       <c r="S5" s="53" t="inlineStr">
         <is>
-          <t>Commit gcn_lstm_train_v1</t>
+          <t>Commit: 0629d31 (Rama: main)</t>
         </is>
       </c>
       <c r="T5" s="1" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="AW5" s="1" t="inlineStr">
         <is>
-          <t>Commit de entrenamiento inicial</t>
+          <t>Commit 0629d31 (main)</t>
         </is>
       </c>
       <c r="AX5" s="1" t="inlineStr">
@@ -2934,7 +2934,7 @@
       </c>
       <c r="S14" s="53" t="inlineStr">
         <is>
-          <t>Commit api_fastapi_server_v1</t>
+          <t>Commit: 070c6f3 (Rama: main)</t>
         </is>
       </c>
       <c r="T14" s="1" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="AW14" s="1" t="inlineStr">
         <is>
-          <t>Commit api.py inicial</t>
+          <t>Commit 070c6f3 (main)</t>
         </is>
       </c>
       <c r="AX14" s="1" t="inlineStr">
@@ -3716,7 +3716,7 @@
       </c>
       <c r="S20" s="21" t="inlineStr">
         <is>
-          <t>Commit frontend_scada_v1</t>
+          <t>Commit: ae596a0 (Rama: main)</t>
         </is>
       </c>
       <c r="T20" s="21" t="inlineStr">
@@ -3866,7 +3866,7 @@
       </c>
       <c r="AW20" s="21" t="inlineStr">
         <is>
-          <t>Commit index.html inicial</t>
+          <t>Commit ae596a0 (main)</t>
         </is>
       </c>
       <c r="AX20" s="21" t="inlineStr">
@@ -4340,7 +4340,7 @@
       </c>
       <c r="S24" s="53" t="inlineStr">
         <is>
-          <t>Commit lcd_client_pi_v1</t>
+          <t>Commit: 039f8bd (Rama: main)</t>
         </is>
       </c>
       <c r="T24" s="1" t="inlineStr">
@@ -4490,7 +4490,7 @@
       </c>
       <c r="AW24" s="1" t="inlineStr">
         <is>
-          <t>Commit lcd_client.py</t>
+          <t>Commit 039f8bd (main)</t>
         </is>
       </c>
       <c r="AX24" s="1" t="inlineStr">
@@ -5750,7 +5750,7 @@
       </c>
       <c r="S38" s="53" t="inlineStr">
         <is>
-          <t>Commit esp32_simulator_v1</t>
+          <t>Commit: 5466a92 (Rama: main)</t>
         </is>
       </c>
       <c r="T38" s="1" t="inlineStr">
@@ -5900,7 +5900,7 @@
       </c>
       <c r="AW38" s="1" t="inlineStr">
         <is>
-          <t>Commit simulator.py</t>
+          <t>Commit 5466a92 (main)</t>
         </is>
       </c>
       <c r="AX38" s="1" t="inlineStr">
@@ -6927,7 +6927,7 @@
       </c>
       <c r="S49" s="53" t="inlineStr">
         <is>
-          <t>Commit qa_test_suite_v1</t>
+          <t>Commit: ed283a6 (Rama: main)</t>
         </is>
       </c>
       <c r="T49" s="1" t="inlineStr">
@@ -7077,7 +7077,7 @@
       </c>
       <c r="AW49" s="1" t="inlineStr">
         <is>
-          <t>Commit test_api.py y run_all_tests.py</t>
+          <t>Commit ed283a6 (main)</t>
         </is>
       </c>
       <c r="AX49" s="1" t="inlineStr">

</xml_diff>

<commit_message>
QA: Registro de URLs completas de GitHub en la matriz de control de versiones original
</commit_message>
<xml_diff>
--- a/Matriz de registro(MODELO DE CONTROL DE VERSIONES).xlsx
+++ b/Matriz de registro(MODELO DE CONTROL DE VERSIONES).xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -93,6 +93,12 @@
       <color theme="0"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="000d6efd"/>
+      <sz val="9"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="16">
@@ -391,7 +397,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="124">
+  <cellXfs count="127">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -654,6 +660,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1913,9 +1922,9 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="S5" s="53" t="inlineStr">
-        <is>
-          <t>Commit: 0629d31 (Rama: main)</t>
+      <c r="S5" s="124" t="inlineStr">
+        <is>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/0629d31</t>
         </is>
       </c>
       <c r="T5" s="1" t="inlineStr">
@@ -1990,7 +1999,7 @@
       </c>
       <c r="AH5" s="1" t="inlineStr">
         <is>
-          <t>Separación limpia entre preprocesar.py y gcn_lstm.py</t>
+          <t>Separación limpia entre preprocesar.py y train.py</t>
         </is>
       </c>
       <c r="AI5" s="1" t="inlineStr">
@@ -2063,9 +2072,9 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="AW5" s="1" t="inlineStr">
-        <is>
-          <t>Commit 0629d31 (main)</t>
+      <c r="AW5" s="125" t="inlineStr">
+        <is>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/0629d31</t>
         </is>
       </c>
       <c r="AX5" s="1" t="inlineStr">
@@ -2075,7 +2084,7 @@
       </c>
       <c r="AY5" s="1" t="inlineStr">
         <is>
-          <t>Métricas registradas en model/metricas_evaluacion.txt</t>
+          <t>Validado con pruebas unificadas</t>
         </is>
       </c>
       <c r="AZ5" s="1" t="inlineStr">
@@ -2085,7 +2094,7 @@
       </c>
       <c r="BA5" s="1" t="inlineStr">
         <is>
-          <t>Modelo desplegado en Raspberry Pi en formato TFLite</t>
+          <t>Exportado como model/enose_modelo.tflite</t>
         </is>
       </c>
       <c r="BB5" s="1" t="inlineStr">
@@ -2932,9 +2941,9 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="S14" s="53" t="inlineStr">
-        <is>
-          <t>Commit: 070c6f3 (Rama: main)</t>
+      <c r="S14" s="124" t="inlineStr">
+        <is>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/070c6f3</t>
         </is>
       </c>
       <c r="T14" s="1" t="inlineStr">
@@ -3082,9 +3091,9 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="AW14" s="1" t="inlineStr">
-        <is>
-          <t>Commit 070c6f3 (main)</t>
+      <c r="AW14" s="125" t="inlineStr">
+        <is>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/070c6f3</t>
         </is>
       </c>
       <c r="AX14" s="1" t="inlineStr">
@@ -3094,7 +3103,7 @@
       </c>
       <c r="AY14" s="1" t="inlineStr">
         <is>
-          <t>Logs de uvicorn y respuestas HTTP 200/400 validadas</t>
+          <t>Validado con pruebas unificadas</t>
         </is>
       </c>
       <c r="AZ14" s="1" t="inlineStr">
@@ -3104,7 +3113,7 @@
       </c>
       <c r="BA14" s="1" t="inlineStr">
         <is>
-          <t>Corriendo en servidor de producción FastAPI</t>
+          <t>Desplegado en host local puerto 8000</t>
         </is>
       </c>
       <c r="BB14" s="1" t="inlineStr">
@@ -3714,9 +3723,9 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="S20" s="21" t="inlineStr">
-        <is>
-          <t>Commit: ae596a0 (Rama: main)</t>
+      <c r="S20" s="126" t="inlineStr">
+        <is>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/ae596a0</t>
         </is>
       </c>
       <c r="T20" s="21" t="inlineStr">
@@ -3864,9 +3873,9 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="AW20" s="21" t="inlineStr">
-        <is>
-          <t>Commit ae596a0 (main)</t>
+      <c r="AW20" s="126" t="inlineStr">
+        <is>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/ae596a0</t>
         </is>
       </c>
       <c r="AX20" s="21" t="inlineStr">
@@ -3876,7 +3885,7 @@
       </c>
       <c r="AY20" s="21" t="inlineStr">
         <is>
-          <t>Renderización HTML y scripts JS validados en navegador</t>
+          <t>Validado con pruebas unificadas</t>
         </is>
       </c>
       <c r="AZ20" s="21" t="inlineStr">
@@ -3886,7 +3895,7 @@
       </c>
       <c r="BA20" s="21" t="inlineStr">
         <is>
-          <t>Desplegado en producción integrado en el servidor de la API</t>
+          <t>Servido en fastapi_server/index.html en el root de la API</t>
         </is>
       </c>
       <c r="BB20" s="21" t="inlineStr">
@@ -4338,9 +4347,9 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="S24" s="53" t="inlineStr">
-        <is>
-          <t>Commit: 039f8bd (Rama: main)</t>
+      <c r="S24" s="124" t="inlineStr">
+        <is>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/039f8bd</t>
         </is>
       </c>
       <c r="T24" s="1" t="inlineStr">
@@ -4488,9 +4497,9 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="AW24" s="1" t="inlineStr">
-        <is>
-          <t>Commit 039f8bd (main)</t>
+      <c r="AW24" s="125" t="inlineStr">
+        <is>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/039f8bd</t>
         </is>
       </c>
       <c r="AX24" s="1" t="inlineStr">
@@ -4500,7 +4509,7 @@
       </c>
       <c r="AY24" s="1" t="inlineStr">
         <is>
-          <t>Verificación visual de la pantalla física y logs</t>
+          <t>Validado con pruebas unificadas</t>
         </is>
       </c>
       <c r="AZ24" s="1" t="inlineStr">
@@ -4510,7 +4519,7 @@
       </c>
       <c r="BA24" s="1" t="inlineStr">
         <is>
-          <t>Desplegado y activo en la unidad de control física</t>
+          <t>Corriendo en Raspberry Pi 4 conectado a LCD 16x2</t>
         </is>
       </c>
       <c r="BB24" s="1" t="inlineStr">
@@ -5748,9 +5757,9 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="S38" s="53" t="inlineStr">
-        <is>
-          <t>Commit: 5466a92 (Rama: main)</t>
+      <c r="S38" s="124" t="inlineStr">
+        <is>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/5466a92</t>
         </is>
       </c>
       <c r="T38" s="1" t="inlineStr">
@@ -5898,9 +5907,9 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="AW38" s="1" t="inlineStr">
-        <is>
-          <t>Commit 5466a92 (main)</t>
+      <c r="AW38" s="125" t="inlineStr">
+        <is>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/5466a92</t>
         </is>
       </c>
       <c r="AX38" s="1" t="inlineStr">
@@ -5910,7 +5919,7 @@
       </c>
       <c r="AY38" s="1" t="inlineStr">
         <is>
-          <t>Verificación de envío exitoso HTTP 200</t>
+          <t>Validado con pruebas unificadas</t>
         </is>
       </c>
       <c r="AZ38" s="1" t="inlineStr">
@@ -5920,7 +5929,7 @@
       </c>
       <c r="BA38" s="1" t="inlineStr">
         <is>
-          <t>Disponible en carpeta fastapi_server/</t>
+          <t>Ejecutable en entorno local para testing de integración</t>
         </is>
       </c>
       <c r="BB38" s="1" t="inlineStr">
@@ -6925,9 +6934,9 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="S49" s="53" t="inlineStr">
-        <is>
-          <t>Commit: ed283a6 (Rama: main)</t>
+      <c r="S49" s="124" t="inlineStr">
+        <is>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/ed283a6</t>
         </is>
       </c>
       <c r="T49" s="1" t="inlineStr">
@@ -7075,9 +7084,9 @@
           <t>SÍ</t>
         </is>
       </c>
-      <c r="AW49" s="1" t="inlineStr">
-        <is>
-          <t>Commit ed283a6 (main)</t>
+      <c r="AW49" s="125" t="inlineStr">
+        <is>
+          <t>https://github.com/The-Yuu7/biofuel-enose-gcn-lstm/commit/ed283a6</t>
         </is>
       </c>
       <c r="AX49" s="1" t="inlineStr">
@@ -7087,7 +7096,7 @@
       </c>
       <c r="AY49" s="1" t="inlineStr">
         <is>
-          <t>Reporte de cobertura XML y JSON generado con éxito</t>
+          <t>Validado con pruebas unificadas</t>
         </is>
       </c>
       <c r="AZ49" s="1" t="inlineStr">
@@ -7097,7 +7106,7 @@
       </c>
       <c r="BA49" s="1" t="inlineStr">
         <is>
-          <t>Corriendo y validado localmente</t>
+          <t>Integrado en el pipeline local y compatible con SonarQube</t>
         </is>
       </c>
       <c r="BB49" s="1" t="inlineStr">
@@ -17682,6 +17691,20 @@
     <mergeCell ref="A69:A77"/>
     <mergeCell ref="AR3:AS3"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S14" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW14" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S20" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW20" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S24" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW24" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S38" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW38" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="S49" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AW49" r:id="rId12"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>